<commit_message>
Initial commit for Streamlit app
</commit_message>
<xml_diff>
--- a/BOM Wall Parts.xlsx
+++ b/BOM Wall Parts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/craignyabvure/Desktop/Python Test Projects AGI/Trailer Loading/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C56401B2-EF6B-094F-91D8-EE7634620252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87B5547-C1F7-F849-851E-89F11AD86CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="3040" windowWidth="27240" windowHeight="16440" xr2:uid="{033D25A6-E8AB-934A-9754-99E28AF88867}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="172">
   <si>
     <t xml:space="preserve">Assembly </t>
   </si>
@@ -444,6 +444,114 @@
   </si>
   <si>
     <t>212078B18</t>
+  </si>
+  <si>
+    <t>198070</t>
+  </si>
+  <si>
+    <t>198071</t>
+  </si>
+  <si>
+    <t>198072</t>
+  </si>
+  <si>
+    <t>198073</t>
+  </si>
+  <si>
+    <t>198074</t>
+  </si>
+  <si>
+    <t>198075</t>
+  </si>
+  <si>
+    <t>198076</t>
+  </si>
+  <si>
+    <t>198077</t>
+  </si>
+  <si>
+    <t>198078</t>
+  </si>
+  <si>
+    <t>198079</t>
+  </si>
+  <si>
+    <t>198080</t>
+  </si>
+  <si>
+    <t>198081</t>
+  </si>
+  <si>
+    <t>198082</t>
+  </si>
+  <si>
+    <t>198083</t>
+  </si>
+  <si>
+    <t>198084</t>
+  </si>
+  <si>
+    <t>198085</t>
+  </si>
+  <si>
+    <t>198086</t>
+  </si>
+  <si>
+    <t>198087</t>
+  </si>
+  <si>
+    <t>198089</t>
+  </si>
+  <si>
+    <t>198090</t>
+  </si>
+  <si>
+    <t>198091</t>
+  </si>
+  <si>
+    <t>198092</t>
+  </si>
+  <si>
+    <t>198093</t>
+  </si>
+  <si>
+    <t>232702B</t>
+  </si>
+  <si>
+    <t>232703C</t>
+  </si>
+  <si>
+    <t>232705E</t>
+  </si>
+  <si>
+    <t>232706F</t>
+  </si>
+  <si>
+    <t>232707G</t>
+  </si>
+  <si>
+    <t>232709J</t>
+  </si>
+  <si>
+    <t>232710K</t>
+  </si>
+  <si>
+    <t>232711L</t>
+  </si>
+  <si>
+    <t>232713U</t>
+  </si>
+  <si>
+    <t>232715W</t>
+  </si>
+  <si>
+    <t>232716X</t>
+  </si>
+  <si>
+    <t>232717Y</t>
+  </si>
+  <si>
+    <t>232719M</t>
   </si>
 </sst>
 </file>
@@ -478,21 +586,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -500,23 +602,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -855,2046 +976,2927 @@
   <dimension ref="A1:D415"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="3" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" style="1" customWidth="1"/>
+    <col min="2" max="3" width="16.33203125" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2">
         <v>194679</v>
       </c>
-      <c r="C2">
-        <v>15</v>
-      </c>
-      <c r="D2">
+      <c r="C2" s="1">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="2">
         <v>194680</v>
       </c>
-      <c r="C3">
-        <v>15</v>
-      </c>
-      <c r="D3">
+      <c r="C3" s="1">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
         <v>194681</v>
       </c>
-      <c r="C4">
-        <v>15</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="1">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="2">
         <v>194682</v>
       </c>
-      <c r="C5">
-        <v>15</v>
-      </c>
-      <c r="D5">
+      <c r="C5" s="1">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>194683</v>
       </c>
-      <c r="C6">
-        <v>15</v>
-      </c>
-      <c r="D6">
+      <c r="C6" s="1">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="2">
         <v>194684</v>
       </c>
-      <c r="C7">
-        <v>15</v>
-      </c>
-      <c r="D7">
+      <c r="C7" s="1">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>194685</v>
       </c>
-      <c r="C8">
-        <v>15</v>
-      </c>
-      <c r="D8">
+      <c r="C8" s="1">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="2">
         <v>194623</v>
       </c>
-      <c r="C9">
-        <v>15</v>
-      </c>
-      <c r="D9">
+      <c r="C9" s="1">
+        <v>15</v>
+      </c>
+      <c r="D9" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>194624</v>
       </c>
-      <c r="C10">
-        <v>15</v>
-      </c>
-      <c r="D10">
+      <c r="C10" s="1">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="2">
         <v>194625</v>
       </c>
-      <c r="C11">
-        <v>15</v>
-      </c>
-      <c r="D11">
+      <c r="C11" s="1">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="2">
         <v>194679</v>
       </c>
-      <c r="C12">
-        <v>15</v>
-      </c>
-      <c r="D12">
+      <c r="C12" s="1">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="2">
         <v>194682</v>
       </c>
-      <c r="C13">
-        <v>15</v>
-      </c>
-      <c r="D13">
+      <c r="C13" s="1">
+        <v>15</v>
+      </c>
+      <c r="D13" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="2">
         <v>194606</v>
       </c>
-      <c r="C14">
-        <v>15</v>
-      </c>
-      <c r="D14">
+      <c r="C14" s="1">
+        <v>15</v>
+      </c>
+      <c r="D14" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="2">
         <v>194607</v>
       </c>
-      <c r="C15">
-        <v>15</v>
-      </c>
-      <c r="D15">
+      <c r="C15" s="1">
+        <v>15</v>
+      </c>
+      <c r="D15" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="2">
         <v>194608</v>
       </c>
-      <c r="C16">
-        <v>15</v>
-      </c>
-      <c r="D16">
+      <c r="C16" s="1">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B17" s="2">
         <v>194604</v>
       </c>
-      <c r="C17">
-        <v>15</v>
-      </c>
-      <c r="D17">
+      <c r="C17" s="1">
+        <v>15</v>
+      </c>
+      <c r="D17" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="2">
         <v>194605</v>
       </c>
-      <c r="C18">
-        <v>15</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="1">
+        <v>15</v>
+      </c>
+      <c r="D18" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B19" s="2">
         <v>194616</v>
       </c>
-      <c r="C19">
-        <v>15</v>
-      </c>
-      <c r="D19">
+      <c r="C19" s="1">
+        <v>15</v>
+      </c>
+      <c r="D19" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="2">
         <v>194617</v>
       </c>
-      <c r="C20">
-        <v>15</v>
-      </c>
-      <c r="D20">
+      <c r="C20" s="1">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="2">
         <v>194618</v>
       </c>
-      <c r="C21">
-        <v>15</v>
-      </c>
-      <c r="D21">
+      <c r="C21" s="1">
+        <v>15</v>
+      </c>
+      <c r="D21" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="2">
         <v>194679</v>
       </c>
-      <c r="C22">
-        <v>15</v>
-      </c>
-      <c r="D22">
+      <c r="C22" s="1">
+        <v>15</v>
+      </c>
+      <c r="D22" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="2">
         <v>194680</v>
       </c>
-      <c r="C23">
-        <v>15</v>
-      </c>
-      <c r="D23">
+      <c r="C23" s="1">
+        <v>15</v>
+      </c>
+      <c r="D23" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="2">
         <v>194681</v>
       </c>
-      <c r="C24">
-        <v>15</v>
-      </c>
-      <c r="D24">
+      <c r="C24" s="1">
+        <v>15</v>
+      </c>
+      <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B25" s="2">
         <v>194682</v>
       </c>
-      <c r="C25">
-        <v>15</v>
-      </c>
-      <c r="D25">
+      <c r="C25" s="1">
+        <v>15</v>
+      </c>
+      <c r="D25" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="2">
         <v>194683</v>
       </c>
-      <c r="C26">
-        <v>15</v>
-      </c>
-      <c r="D26">
+      <c r="C26" s="1">
+        <v>15</v>
+      </c>
+      <c r="D26" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B27" s="2">
         <v>194684</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="1">
         <v>18</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="2">
         <v>194623</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="1">
         <v>18</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="A29" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B29" s="2">
         <v>194624</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="1">
         <v>18</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="A30" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="2">
         <v>194625</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="1">
         <v>18</v>
       </c>
-      <c r="D30">
+      <c r="D30" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="A31" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B31" s="2">
         <v>194685</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="1">
         <v>18</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="A32" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="2">
         <v>194679</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="1">
         <v>18</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="A33" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B33" s="2">
         <v>194680</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="1">
         <v>18</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="A34" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="2">
         <v>194681</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="1">
         <v>18</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="A35" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B35" s="2">
         <v>194682</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="1">
         <v>18</v>
       </c>
-      <c r="D35">
+      <c r="D35" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="A36" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="2">
         <v>194683</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="1">
         <v>18</v>
       </c>
-      <c r="D36">
+      <c r="D36" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="A37" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B37" s="2">
         <v>194684</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="1">
         <v>18</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>15</v>
-      </c>
-      <c r="B38" s="1">
+      <c r="A38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B38" s="2">
         <v>194623</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="1">
         <v>18</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="A39" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B39" s="2">
         <v>194624</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="1">
         <v>18</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>15</v>
-      </c>
-      <c r="B40" s="1">
+      <c r="A40" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="2">
         <v>194625</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="1">
         <v>18</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="A41" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B41" s="2">
         <v>194679</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="1">
         <v>18</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="A42" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="2">
         <v>194680</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="1">
         <v>18</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="A43" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B43" s="2">
         <v>194681</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="1">
         <v>18</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="2">
         <v>194682</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="1">
         <v>18</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="A45" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B45" s="2">
         <v>194683</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="1">
         <v>18</v>
       </c>
-      <c r="D45">
+      <c r="D45" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="A46" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="2">
         <v>194684</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="1">
         <v>18</v>
       </c>
-      <c r="D46">
+      <c r="D46" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="A47" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B47" s="2">
         <v>194623</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="1">
         <v>18</v>
       </c>
-      <c r="D47">
+      <c r="D47" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="A48" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="2">
         <v>194624</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="1">
         <v>18</v>
       </c>
-      <c r="D48">
+      <c r="D48" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="A49" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B49" s="2">
         <v>194625</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="1">
         <v>18</v>
       </c>
-      <c r="D49">
+      <c r="D49" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="A50" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="4">
+      <c r="B50" s="3">
         <v>194920</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="1">
         <v>21</v>
       </c>
-      <c r="D50">
+      <c r="D50" s="1">
         <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="A51" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B51" s="4">
+      <c r="B51" s="3">
         <v>194921</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="1">
         <v>21</v>
       </c>
-      <c r="D51">
+      <c r="D51" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="A52" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B52" s="4">
+      <c r="B52" s="3">
         <v>194922</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="1">
         <v>21</v>
       </c>
-      <c r="D52">
+      <c r="D52" s="1">
         <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="A53" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B53" s="4">
+      <c r="B53" s="3">
         <v>194923</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="1">
         <v>21</v>
       </c>
-      <c r="D53">
+      <c r="D53" s="1">
         <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="A54" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B54" s="4">
+      <c r="B54" s="3">
         <v>194925</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="1">
         <v>21</v>
       </c>
-      <c r="D54">
+      <c r="D54" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+      <c r="A55" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B55" s="4">
+      <c r="B55" s="3">
         <v>194950</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="1">
         <v>21</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+      <c r="A56" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B56" s="4">
+      <c r="B56" s="3">
         <v>194951</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="1">
         <v>21</v>
       </c>
-      <c r="D56">
+      <c r="D56" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="A57" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B57" s="4">
+      <c r="B57" s="3">
         <v>194952</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="1">
         <v>21</v>
       </c>
-      <c r="D57">
+      <c r="D57" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="A58" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B58" s="4">
+      <c r="B58" s="3">
         <v>194953</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="1">
         <v>21</v>
       </c>
-      <c r="D58">
+      <c r="D58" s="1">
         <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="A59" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B59" s="4">
+      <c r="B59" s="3">
         <v>194954</v>
       </c>
-      <c r="C59">
+      <c r="C59" s="1">
         <v>21</v>
       </c>
-      <c r="D59">
+      <c r="D59" s="1">
         <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+      <c r="A60" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B60" s="4">
+      <c r="B60" s="3">
         <v>194955</v>
       </c>
-      <c r="C60">
+      <c r="C60" s="1">
         <v>21</v>
       </c>
-      <c r="D60">
+      <c r="D60" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+      <c r="A61" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B61" s="4">
+      <c r="B61" s="3">
         <v>194956</v>
       </c>
-      <c r="C61">
+      <c r="C61" s="1">
         <v>21</v>
       </c>
-      <c r="D61">
+      <c r="D61" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+      <c r="A62" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B62" s="4">
+      <c r="B62" s="3">
         <v>194957</v>
       </c>
-      <c r="C62">
+      <c r="C62" s="1">
         <v>21</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="1">
         <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+      <c r="A63" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B63" s="4">
+      <c r="B63" s="3">
         <v>194971</v>
       </c>
-      <c r="C63">
+      <c r="C63" s="1">
         <v>21</v>
       </c>
-      <c r="D63">
+      <c r="D63" s="1">
         <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+      <c r="A64" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B64" s="4">
+      <c r="B64" s="3">
         <v>194978</v>
       </c>
-      <c r="C64">
+      <c r="C64" s="1">
         <v>21</v>
       </c>
-      <c r="D64">
+      <c r="D64" s="1">
         <v>4</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+      <c r="A65" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B65" s="4">
+      <c r="B65" s="3">
         <v>194978</v>
       </c>
-      <c r="C65">
+      <c r="C65" s="1">
         <v>21</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+      <c r="A66" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B66" s="4">
+      <c r="B66" s="3">
         <v>194990</v>
       </c>
-      <c r="C66">
+      <c r="C66" s="1">
         <v>21</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="1">
         <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+      <c r="A67" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B67" s="4">
+      <c r="B67" s="3">
         <v>194991</v>
       </c>
-      <c r="C67">
+      <c r="C67" s="1">
         <v>21</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+      <c r="A68" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B68" s="4">
+      <c r="B68" s="3">
         <v>194992</v>
       </c>
-      <c r="C68">
+      <c r="C68" s="1">
         <v>21</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="A69" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B69" s="4">
+      <c r="B69" s="3">
         <v>194993</v>
       </c>
-      <c r="C69">
+      <c r="C69" s="1">
         <v>21</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="A70" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B70" s="4">
+      <c r="B70" s="3">
         <v>194994</v>
       </c>
-      <c r="C70">
+      <c r="C70" s="1">
         <v>21</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="1">
         <v>7</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+      <c r="A71" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B71" s="4">
+      <c r="B71" s="3">
         <v>194995</v>
       </c>
-      <c r="C71">
+      <c r="C71" s="1">
         <v>21</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="1">
         <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+      <c r="A72" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B72" s="4">
+      <c r="B72" s="3">
         <v>194996</v>
       </c>
-      <c r="C72">
+      <c r="C72" s="1">
         <v>21</v>
       </c>
-      <c r="D72">
+      <c r="D72" s="1">
         <v>7</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B73" s="4">
+      <c r="A73" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B73" s="3">
         <v>235301</v>
       </c>
-      <c r="C73">
+      <c r="C73" s="1">
         <v>21</v>
       </c>
-      <c r="D73">
+      <c r="D73" s="1">
         <v>6</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B74" t="s">
+      <c r="A74" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B74" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D74">
+      <c r="D74" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B75" t="s">
+      <c r="A75" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B75" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D75">
+      <c r="D75" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B76" t="s">
+      <c r="A76" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B76" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B77" t="s">
+      <c r="A77" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B77" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D77">
+      <c r="D77" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B78" t="s">
+      <c r="A78" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B78" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D78">
+      <c r="D78" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B79" t="s">
+      <c r="A79" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D79">
+      <c r="D79" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B80" t="s">
+      <c r="A80" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D80">
+      <c r="D80" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B81" t="s">
+      <c r="A81" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B81" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D81">
+      <c r="D81" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B82" t="s">
+      <c r="A82" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B82" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D82">
+      <c r="D82" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B83" t="s">
+      <c r="A83" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B83" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D83">
+      <c r="D83" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B84" t="s">
+      <c r="A84" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B84" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D84">
+      <c r="D84" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B85" t="s">
+      <c r="A85" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B85" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D85">
+      <c r="D85" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B86" t="s">
+      <c r="A86" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D86">
+      <c r="D86" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B87" t="s">
+      <c r="A87" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B87" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D87">
+      <c r="D87" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B88" t="s">
+      <c r="A88" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B88" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D88">
+      <c r="D88" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B89" t="s">
+      <c r="A89" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B89" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D89">
+      <c r="D89" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B90" t="s">
+      <c r="A90" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B90" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B91" t="s">
+      <c r="A91" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B91" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D91">
+      <c r="D91" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B92" t="s">
+      <c r="A92" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B92" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D92">
+      <c r="D92" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B93" t="s">
+      <c r="A93" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B93" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D93">
+      <c r="D93" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B94" t="s">
+      <c r="A94" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B94" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D94">
+      <c r="D94" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B95" t="s">
+      <c r="A95" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B95" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D95">
+      <c r="D95" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B96" t="s">
+      <c r="A96" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B96" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D96">
+      <c r="D96" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B97" t="s">
+      <c r="A97" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B97" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D97">
+      <c r="D97" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B98" t="s">
+      <c r="A98" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B98" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D98">
+      <c r="D98" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B99" t="s">
+      <c r="A99" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B99" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D99">
+      <c r="D99" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B100" t="s">
+      <c r="A100" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B101" t="s">
+      <c r="A101" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D101">
+      <c r="D101" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B102" t="s">
+      <c r="A102" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B102" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D102">
+      <c r="D102" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A103" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B103" t="s">
+      <c r="A103" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B103" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D103">
+      <c r="D103" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A104" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B104" t="s">
+      <c r="A104" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B104" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D104">
+      <c r="D104" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A105" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B105" t="s">
+      <c r="A105" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B105" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D105">
+      <c r="D105" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A106" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B106" t="s">
+      <c r="A106" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B106" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A107" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B107" t="s">
+      <c r="A107" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B107" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D107">
+      <c r="D107" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A108" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B108" t="s">
+      <c r="A108" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B108" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D108">
+      <c r="D108" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A109" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B109" t="s">
+      <c r="A109" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B109" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D109">
+      <c r="D109" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A110" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B110" t="s">
+      <c r="A110" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B110" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D110">
+      <c r="D110" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A111" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B111" t="s">
+      <c r="A111" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B111" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D111">
+      <c r="D111" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A112" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B112" t="s">
+      <c r="A112" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B112" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D112">
+      <c r="D112" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A113" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B113" t="s">
+      <c r="A113" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B113" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D113">
+      <c r="D113" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A114" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B114" t="s">
+      <c r="A114" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B114" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D114">
+      <c r="D114" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A115" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B115" t="s">
+      <c r="A115" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B115" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D115">
+      <c r="D115" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A116" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B116" t="s">
+      <c r="A116" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B116" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D116">
+      <c r="D116" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A117" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B117" t="s">
+      <c r="A117" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B117" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D117">
+      <c r="D117" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A118" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B118" t="s">
+      <c r="A118" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B118" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D118">
+      <c r="D118" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A119" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B119" t="s">
+      <c r="A119" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B119" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D119">
+      <c r="D119" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A120" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B120" t="s">
+      <c r="A120" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B120" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D120">
+      <c r="D120" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A121" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B121" t="s">
+      <c r="A121" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B121" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D121">
+      <c r="D121" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A122" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B122" t="s">
+      <c r="A122" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B122" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D122">
+      <c r="D122" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A123" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B123" t="s">
+      <c r="A123" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B123" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D123">
+      <c r="D123" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A124" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B124" t="s">
+      <c r="A124" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B124" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D124">
+      <c r="D124" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A125" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B125" t="s">
+      <c r="A125" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B125" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D125">
+      <c r="D125" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A126" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B126" t="s">
+      <c r="A126" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B126" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D126">
+      <c r="D126" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B127" t="s">
+      <c r="A127" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B127" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D127">
+      <c r="D127" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B128" t="s">
+      <c r="A128" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B128" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D128">
+      <c r="D128" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B129" t="s">
+      <c r="A129" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B129" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D129">
+      <c r="D129" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B130" t="s">
+      <c r="A130" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B130" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D130">
+      <c r="D130" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A131" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B131" t="s">
+      <c r="A131" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B131" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D131">
+      <c r="D131" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A132" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B132" t="s">
+      <c r="A132" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B132" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D132">
+      <c r="D132" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A133" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B133" t="s">
+      <c r="A133" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B133" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D133">
+      <c r="D133" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A134" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B134" t="s">
+      <c r="A134" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B134" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="D134">
+      <c r="D134" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A135" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B135" t="s">
+      <c r="A135" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B135" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D135">
+      <c r="D135" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A136" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B136" t="s">
+      <c r="A136" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B136" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D136">
+      <c r="D136" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A137" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B137" t="s">
+      <c r="A137" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B137" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D137">
+      <c r="D137" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A138" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B138" t="s">
+      <c r="A138" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B138" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="D138">
+      <c r="D138" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A139" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B139" t="s">
+      <c r="A139" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B139" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D139">
+      <c r="D139" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A140" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B140" t="s">
+      <c r="A140" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B140" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D140">
+      <c r="D140" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A141" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B141" t="s">
+      <c r="A141" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B141" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D141">
+      <c r="D141" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A142" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B142" t="s">
+      <c r="A142" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B142" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D142">
+      <c r="D142" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A143" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B143" t="s">
+      <c r="A143" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B143" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D143">
+      <c r="D143" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A144" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B144" t="s">
+      <c r="A144" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B144" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D144">
+      <c r="D144" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A145" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B145" t="s">
+      <c r="A145" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B145" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D145">
+      <c r="D145" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A146" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B146" t="s">
+      <c r="A146" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B146" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D146">
+      <c r="D146" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A147" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B147" t="s">
+      <c r="A147" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B147" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D147">
+      <c r="D147" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A148" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B148" t="s">
+      <c r="A148" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B148" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D148">
+      <c r="D148" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A149" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B149" t="s">
+      <c r="A149" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B149" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D149">
+      <c r="D149" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A150" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B150" t="s">
+      <c r="A150" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B150" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D150">
+      <c r="D150" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A151" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B151" t="s">
+      <c r="A151" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B151" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D151">
+      <c r="D151" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A152" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B152" t="s">
+      <c r="A152" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B152" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D152">
+      <c r="D152" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A153" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B153" t="s">
+      <c r="A153" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B153" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D153">
+      <c r="D153" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A154" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B154" t="s">
+      <c r="A154" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B154" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D154">
+      <c r="D154" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A155" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B155" t="s">
+      <c r="A155" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B155" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D155">
+      <c r="D155" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A156" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B156" t="s">
+      <c r="A156" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B156" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D156">
+      <c r="D156" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A157" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B157" t="s">
+      <c r="A157" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B157" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D157">
+      <c r="D157" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A158" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B158" t="s">
+      <c r="A158" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B158" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D158">
+      <c r="D158" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A159" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B159" t="s">
+      <c r="A159" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B159" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D159">
+      <c r="D159" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A160" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B160" t="s">
+      <c r="A160" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B160" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D160">
+      <c r="D160" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A161" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B161" t="s">
+      <c r="A161" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B161" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D161">
+      <c r="D161" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A162" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B162" t="s">
+      <c r="A162" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B162" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D162">
+      <c r="D162" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A163" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B163" t="s">
+      <c r="A163" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B163" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D163">
+      <c r="D163" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A164" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B164" t="s">
+      <c r="A164" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B164" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D164">
+      <c r="D164" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A165" s="3">
-        <v>233254</v>
-      </c>
-      <c r="B165" t="s">
+      <c r="A165" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B165" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D165">
-        <v>2</v>
+      <c r="D165" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A166" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D166" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A167" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D167" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A168" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D168" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A169" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D169" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A170" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D170" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A171" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D171" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A172" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D172" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A173" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D173" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A174" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D174" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A175" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D175" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A176" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B176" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D176" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A177" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D177" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A178" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D178" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A179" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D179" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A180" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D180" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A181" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B181" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D181" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A182" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B182" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="D182" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A183" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B183" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D183" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A184" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D184" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A185" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B185" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D185" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A186" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D186" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A187" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D187" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A188" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D188" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A189" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B189" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D189" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A190" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D190" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A191" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D191" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A192" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D192" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A193" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D193" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A194" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D194" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A195" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D195" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A196" s="4">
+        <v>233254</v>
+      </c>
+      <c r="B196" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D196" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A197" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B197" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D197" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A198" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B198" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D198" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A199" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B199" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D199" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A200" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B200" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D200" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A201" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B201" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D201" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A202" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B202" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D202" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A203" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B203" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D203" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A204" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B204" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D204" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A205" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B205" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D205" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A206" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B206" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D206" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A207" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B207" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D207" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A208" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B208" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D208" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A209" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B209" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D209" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A210" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B210" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D210" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A211" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B211" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D211" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A212" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B212" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D212" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A213" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B213" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D213" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A214" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B214" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D214" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A215" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B215" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D215" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A216" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B216" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D216" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A217" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B217" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D217" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A218" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B218" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D218" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A219" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B219" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D219" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A220" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B220" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D220" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A221" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B221" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D221" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A222" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B222" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D222" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A223" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B223" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D223" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A224" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B224" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D224" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A225" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B225" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D225" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A226" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B226" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D226" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A227" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B227" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D227" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A228" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B228" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D228" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A229" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B229" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D229" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A230" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B230" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D230" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A231" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B231" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D231" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A232" s="4">
+        <v>4446667</v>
+      </c>
+      <c r="B232" s="4">
+        <v>333333</v>
+      </c>
+      <c r="D232" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A233" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B233" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D233" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="234" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A234" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B234" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D234" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="235" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A235" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B235" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D235" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="236" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A236" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B236" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D236" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A237" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B237" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D237" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="238" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A238" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B238" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D238" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A239" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B239" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D239" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A240" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B240" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D240" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A241" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B241" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D241" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="242" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A242" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B242" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D242" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="243" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A243" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B243" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D243" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="244" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A244" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B244" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D244" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="245" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A245" s="4">
+        <v>78986</v>
+      </c>
+      <c r="B245" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D245" s="1">
+        <v>15</v>
       </c>
     </row>
     <row r="415" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B415" s="3"/>
+      <c r="B415" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>